<commit_message>
📊 Horarios actualizados Línea 141 - 2596
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,141 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:39:02</t>
+          <t>Última actualización: 02:50:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>02:50:55</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>02:51</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02:50:55</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>03:48</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>58</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:50:55</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>71</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>02:50:55</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:37</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>107</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -454,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,14 +594,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:39:02</t>
+          <t>Última actualización: 02:50:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>02:50:55</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>02:51</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02:50:55</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>04:37</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>107</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -502,7 +706,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:39:02</t>
+          <t>Última actualización: 02:50:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2597
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:50:55</t>
+          <t>Última actualización: 04:19:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:50:55</t>
+          <t>04:19:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:51</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:50:55</t>
+          <t>04:19:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:50:55</t>
+          <t>04:19:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,23 +548,173 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>02:50:55</t>
+          <t>04:19:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:37</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:34</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>75</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:34</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>75</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:46</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>87</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:04</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>105</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>112</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>115</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -581,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,14 +744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:50:55</t>
+          <t>Última actualización: 04:19:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -635,21 +785,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:50:55</t>
+          <t>04:19:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:51</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -660,23 +810,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:50:55</t>
+          <t>04:19:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:37</t>
+          <t>05:34</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>112</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -693,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -706,14 +881,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:50:55</t>
+          <t>Última actualización: 04:19:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>05:43</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>84</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:19:40</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>112</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2598
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:19:40</t>
+          <t>Última actualización: 06:06:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:19:40</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>112</v>
+        <v>5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:19:40</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -712,9 +712,559 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>115</v>
+        <v>8</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:21</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:24</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>86XR36_ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>18</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:27</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>21</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>24</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>25</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>06:44</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>38</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>06:47</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>41</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>54</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07:01</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>55</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>10_RUTA 36_ESC 70</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>56</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07:05</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>59</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07:07</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>61</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>65</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>75</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>86</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>86</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>07:34</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>88</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>91</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>102</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>105</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>106</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>08:04</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>118</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -731,7 +1281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,14 +1294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:19:40</t>
+          <t>Última actualización: 06:06:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -835,7 +1385,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:19:40</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -849,9 +1399,84 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>112</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>41</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>65</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>106</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -868,7 +1493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -881,14 +1506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:19:40</t>
+          <t>Última actualización: 06:06:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -964,6 +1589,106 @@
         <v>112</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>54</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>85</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2599
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:06:13</t>
+          <t>Última actualización: 07:40:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>07:48</t>
+          <t>07:42</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>102</v>
+        <v>2</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:47</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>105</v>
+        <v>7</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>07:52</t>
+          <t>07:48</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>106</v>
+        <v>8</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1253,18 +1253,643 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>105</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>11</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>106</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>15</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>19</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>20</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>08:03</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>23</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>08:04</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D44" t="n">
         <v>118</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>08:12</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>32</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>08:13</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>33</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>41</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>43</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>43</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>08:27</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>47</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>08:42</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>62</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>64</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>08:57</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>77</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>91</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>91</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>97</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>101</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>101</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>103</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>104</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>09:32</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>112</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>113</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1281,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1294,14 +1919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:06:13</t>
+          <t>Última actualización: 07:40:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1460,23 +2085,98 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>11</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:06:13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>07:52</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215D_EL PATO</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>106</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>43</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>91</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1493,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1506,14 +2206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:06:13</t>
+          <t>Última actualización: 07:40:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1691,6 +2391,106 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>40</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>60</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07:40:17</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>87</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2600
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:17</t>
+          <t>Última actualización: 08:43:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 73</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>08:57</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>77</v>
+        <v>1</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>08:53</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>91</v>
+        <v>10</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>97</v>
+        <v>21</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>101</v>
+        <v>22</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>09:23</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>103</v>
+        <v>28</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>104</v>
+        <v>29</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>09:32</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>112</v>
+        <v>30</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,23 +1873,423 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>34</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>38</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>38</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>07:40:17</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>103</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>40</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>41</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>09:32</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>49</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
         <is>
           <t>09:33</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D62" t="n">
-        <v>113</v>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="D69" t="n">
+        <v>50</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>52</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>57</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>59</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>61</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>09:52</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>69</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>88</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>98</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>104</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>119</v>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1906,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1919,14 +2319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:17</t>
+          <t>Última actualización: 08:43:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2177,6 +2577,81 @@
         <v>91</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:12</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>29</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>59</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>104</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2193,7 +2668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2206,14 +2681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:40:17</t>
+          <t>Última actualización: 08:43:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2472,25 +2947,100 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>9</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>07:40:17</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>09:07</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>215D_LA PLATA</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D16" t="n">
         <v>87</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>32</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>80</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2601
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:43:14</t>
+          <t>Última actualización: 09:46:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 73</t>
+          <t>Total filas: 100</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>09:46:33</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:52</t>
+          <t>09:46</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,12 +2198,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>09:46:33</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:47</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>09:46:33</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>98</v>
+        <v>6</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>09:46:33</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>104</v>
+        <v>17</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,23 +2273,698 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>18</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>24</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>08:43:14</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>88</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>26</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>27</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>35</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>36</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>36</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>10:23</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>37</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>40</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>08:43:14</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>104</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>47</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>48</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>48</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
         <is>
           <t>10:42</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D78" t="n">
-        <v>119</v>
-      </c>
-      <c r="E78" t="inlineStr">
+      <c r="D92" t="n">
+        <v>56</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>57</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>66</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>70</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>76</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>80</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>11:09</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>83</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>10_ESC70-OLMOS</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>85</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>11:14</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>88</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>93</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>95</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>106</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>112</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>116</v>
+      </c>
+      <c r="E105" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2306,7 +2981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2319,14 +2994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:43:14</t>
+          <t>Última actualización: 09:46:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2635,23 +3310,73 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>08:43:14</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>10:27</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>104</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>76</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2668,7 +3393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2681,14 +3406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:43:14</t>
+          <t>Última actualización: 09:46:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3747,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>09:46:33</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3036,11 +3761,61 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:47</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>61</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>82</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2602
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E105"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:46:33</t>
+          <t>Última actualización: 11:21:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 100</t>
+          <t>Total filas: 127</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>09:46:33</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>09:46:33</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:22</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>106</v>
+        <v>1</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:46:33</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>112</v>
+        <v>11</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,23 +2948,698 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>13</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>14</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>16</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
           <t>09:46:33</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>112</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>20</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>09:46:33</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
         <is>
           <t>11:42</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D105" t="n">
+      <c r="D110" t="n">
         <v>116</v>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>11:51</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>30</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>31</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>31</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>10_ESC70-OLMOS</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>33</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>12:02</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>84_ESC AGRARIA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>41</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>43</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>45</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>45</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>49</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>12:12</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>51</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>57</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>59</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>59</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>59</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>73</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>73</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>75</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>79</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>12:48</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>87</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>104</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>104</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>105</v>
+      </c>
+      <c r="E132" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2981,7 +3656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2994,14 +3669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:46:33</t>
+          <t>Última actualización: 11:21:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3377,6 +4052,81 @@
         <v>76</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:51</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>30</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>59</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>104</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3393,7 +4143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3406,14 +4156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:46:33</t>
+          <t>Última actualización: 11:21:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3814,6 +4564,56 @@
         <v>82</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:02</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>41</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>92</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2603
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E132"/>
+  <dimension ref="A1:E156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:21:53</t>
+          <t>Última actualización: 12:48:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 127</t>
+          <t>Total filas: 151</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>104</v>
+        <v>1</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>104</v>
+        <v>1</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,23 +3623,623 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>2</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>7</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>15</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>17</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
           <t>11:21:53</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>104</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>104</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
         <is>
           <t>13:06</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr">
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>18</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>11:21:53</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D132" t="n">
+      <c r="D139" t="n">
         <v>105</v>
       </c>
-      <c r="E132" t="inlineStr">
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>19</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>13:08</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>20</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>27</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>13:16</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>28</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>33</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>35</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>38</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>13:27</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>39</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>47</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>47</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>63</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>68</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>69</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>89</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>89</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>92</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>100</v>
+      </c>
+      <c r="E156" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3656,7 +4256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3669,14 +4269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:21:53</t>
+          <t>Última actualización: 12:48:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4127,6 +4727,81 @@
         <v>104</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:06</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>18</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>63</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>92</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4143,7 +4818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4156,14 +4831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:21:53</t>
+          <t>Última actualización: 12:48:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4597,25 +5272,100 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>11:21:53</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>12:53</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D23" t="n">
         <v>92</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>43</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>69</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2604
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E156"/>
+  <dimension ref="A1:E183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:15</t>
+          <t>Última actualización: 13:42:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 151</t>
+          <t>Total filas: 178</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>104</v>
+        <v>17</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>18</v>
+        <v>105</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3808,11 +3808,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>105</v>
+        <v>18</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:42</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:43</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>13:57</t>
+          <t>13:43</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>89</v>
+        <v>3</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:46</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>89</v>
+        <v>4</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>14:20</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,23 +4223,698 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>8</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
           <t>12:48:15</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>63</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>13</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>14</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>68</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>69</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>20</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>22</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>22</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>34</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>34</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>89</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>89</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>37</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>92</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>39</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
         <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
+      <c r="C172" t="inlineStr">
         <is>
           <t>26_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D156" t="n">
+      <c r="D172" t="n">
         <v>100</v>
       </c>
-      <c r="E156" t="inlineStr">
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>48</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>52</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>62</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>74</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>76</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>78</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>83</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>98</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>103</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>108</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>112</v>
+      </c>
+      <c r="E183" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4256,7 +4931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4269,14 +4944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:15</t>
+          <t>Última actualización: 13:42:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4760,12 +5435,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4774,7 +5449,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>63</v>
+        <v>8</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4790,18 +5465,118 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>63</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>37</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:48:15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>14:20</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D27" t="n">
         <v>92</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>76</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>112</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4818,7 +5593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4831,14 +5606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:15</t>
+          <t>Última actualización: 13:42:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -5364,6 +6139,81 @@
         <v>69</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>19</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>65</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>105</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2605
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E183"/>
+  <dimension ref="A1:E208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:48</t>
+          <t>Última actualización: 14:43:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 178</t>
+          <t>Total filas: 203</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>76</v>
+        <v>1</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,12 +4798,12 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,12 +4823,12 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>103</v>
+        <v>4</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:52</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>108</v>
+        <v>9</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4903,18 +4903,643 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>74</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>14</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>15</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>17</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>22</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>22</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>27</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>30</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>37</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>38</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>103</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>47</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
           <t>15:34</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
+      <c r="C195" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D183" t="n">
+      <c r="D195" t="n">
         <v>112</v>
       </c>
-      <c r="E183" t="inlineStr">
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>52</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>15:43</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>60</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>64</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>64</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>15:50</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>67</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>72</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>74</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>92</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>97</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>100</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>104</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>10_ESC70-OLMOS</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>106</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>114</v>
+      </c>
+      <c r="E208" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4931,7 +5556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4944,14 +5569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:48</t>
+          <t>Última actualización: 14:43:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -5535,7 +6160,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5549,7 +6174,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5577,6 +6202,56 @@
         <v>112</v>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>52</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>97</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5593,7 +6268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5606,14 +6281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:48</t>
+          <t>Última actualización: 14:43:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -6172,12 +6847,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -6186,7 +6861,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -6202,20 +6877,95 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>65</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:42:48</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>15:27</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D29" t="n">
         <v>105</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>47</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>16:08</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>85</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2606
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E208"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:43:05</t>
+          <t>Última actualización: 15:45:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 203</t>
+          <t>Total filas: 231</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:46</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>15:46</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5353,16 +5353,16 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>74</v>
+        <v>2</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>92</v>
+        <v>5</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>104</v>
+        <v>15</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>16:29</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>10_ESC70-OLMOS</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>106</v>
+        <v>16</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,23 +5523,723 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>20</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>25</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>30</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>35</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>16:21</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>36</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>16:22</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>37</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
           <t>14:43:05</t>
         </is>
       </c>
-      <c r="B208" t="inlineStr">
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>100</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>104</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>10_ESC70-OLMOS</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>44</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>45</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>16:36</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>51</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>14:43:05</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
         <is>
           <t>16:37</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
+      <c r="C219" t="inlineStr">
         <is>
           <t>11_ESC 3-ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D208" t="n">
+      <c r="D219" t="n">
         <v>114</v>
       </c>
-      <c r="E208" t="inlineStr">
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>55</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>57</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>58</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>65</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>71</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>16:57</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>72</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>16:58</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>73</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>76</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>79</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>17:12</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>87</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>17:16</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>91</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>96</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>97</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>99</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>17:28</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>103</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>112</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>115</v>
+      </c>
+      <c r="E236" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5556,7 +6256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5569,14 +6269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:43:05</t>
+          <t>Última actualización: 15:45:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -6235,7 +6935,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6249,9 +6949,59 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>97</v>
+        <v>35</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>79</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>115</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6268,7 +7018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6281,14 +7031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:43:05</t>
+          <t>Última actualización: 15:45:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -6947,7 +7697,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6961,11 +7711,61 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>74</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2607
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:45:19</t>
+          <t>Última actualización: 16:51:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 231</t>
+          <t>Total filas: 251</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>104</v>
+        <v>17</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>71</v>
+        <v>5</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,7 +5948,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>72</v>
+        <v>6</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,16 +6028,16 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>87</v>
+        <v>12</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6078,16 +6078,16 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>17:16</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>97</v>
+        <v>19</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6153,16 +6153,16 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6178,16 +6178,16 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>17:28</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:17</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>112</v>
+        <v>26</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,23 +6223,523 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>30</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>30</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
           <t>15:45:19</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>97</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>33</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>15:45:19</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>17:28</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>103</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>17:29</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>38</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>40</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>44</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>46</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
         <is>
           <t>17:40</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
+      <c r="C245" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D236" t="n">
-        <v>115</v>
-      </c>
-      <c r="E236" t="inlineStr">
+      <c r="D245" t="n">
+        <v>49</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>17:46</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>55</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>17:46</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>55</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>60</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>61</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>74</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>18:07</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>76</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>92</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>93</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>103</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>108</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>109</v>
+      </c>
+      <c r="E256" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6256,7 +6756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6269,14 +6769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:45:19</t>
+          <t>Última actualización: 16:51:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6985,23 +7485,73 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>14</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>17:40</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>115</v>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D34" t="n">
+        <v>49</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>92</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7018,7 +7568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7031,14 +7581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:45:19</t>
+          <t>Última actualización: 16:51:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -7722,7 +8272,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7736,7 +8286,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -7764,6 +8314,81 @@
         <v>100</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>47</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:58</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>67</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>109</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2608
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E256"/>
+  <dimension ref="A1:E278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:51:15</t>
+          <t>Última actualización: 17:38:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 251</t>
+          <t>Total filas: 273</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>10</v>
+        <v>76</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>17:46</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>17:46</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>60</v>
+        <v>3</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6578,16 +6578,16 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:46</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>18:07</t>
+          <t>17:46</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -6612,7 +6612,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6653,16 +6653,16 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>93</v>
+        <v>60</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>103</v>
+        <v>14</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>108</v>
+        <v>17</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,23 +6723,573 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>17:58</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>20</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>22</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>26</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>26</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
           <t>16:51:15</t>
         </is>
       </c>
-      <c r="B256" t="inlineStr">
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>74</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>18:07</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>29</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>43</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>44</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>92</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>93</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>56</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>108</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
         <is>
           <t>18:40</t>
         </is>
       </c>
-      <c r="C256" t="inlineStr">
+      <c r="C268" t="inlineStr">
         <is>
           <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
-      <c r="D256" t="n">
-        <v>109</v>
-      </c>
-      <c r="E256" t="inlineStr">
+      <c r="D268" t="n">
+        <v>62</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>62</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>66</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>18:57</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>79</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>86</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>19:06</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>88</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>19:10</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>92</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>98</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>110</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>112</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>118</v>
+      </c>
+      <c r="E278" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6756,7 +7306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6769,14 +7319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:51:15</t>
+          <t>Última actualización: 17:38:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -7510,7 +8060,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7524,7 +8074,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -7535,23 +8085,73 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>44</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>16:51:15</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D36" t="n">
         <v>92</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:57</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>79</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7568,7 +8168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7581,14 +8181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:51:15</t>
+          <t>Última actualización: 17:38:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -8322,7 +8922,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8336,7 +8936,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -8347,12 +8947,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>17:58</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -8361,7 +8961,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -8377,18 +8977,93 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>17:58</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>67</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:51:15</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>18:40</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D37" t="n">
         <v>109</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>64</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19:10</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>92</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2609
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E278"/>
+  <dimension ref="A1:E300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:38:48</t>
+          <t>Última actualización: 18:26:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 273</t>
+          <t>Total filas: 295</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>06:06:13</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:06:13</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>104</v>
+        <v>17</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>105</v>
+        <v>18</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3808,11 +3808,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>18</v>
+        <v>105</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:28</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:29</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_ESC70-OLMOS</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>108</v>
+        <v>3</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>62</v>
+        <v>4</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>18:57</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>79</v>
+        <v>8</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,12 +7123,12 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -7137,7 +7137,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>19:06</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:43</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>98</v>
+        <v>17</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7228,16 +7228,16 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>112</v>
+        <v>20</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,23 +7273,573 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>18:57</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>31</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>34</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
           <t>17:38:48</t>
         </is>
       </c>
-      <c r="B278" t="inlineStr">
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>86</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>38</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>19:06</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>40</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>19:10</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>92</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>45</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>50</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>53</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>55</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>61</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>110</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>64</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
         <is>
           <t>19:36</t>
         </is>
       </c>
-      <c r="C278" t="inlineStr">
+      <c r="C291" t="inlineStr">
         <is>
           <t>26_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D278" t="n">
+      <c r="D291" t="n">
         <v>118</v>
       </c>
-      <c r="E278" t="inlineStr">
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>19:42</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>76</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>80</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>85</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>19:52</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>86</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>19:59</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>93</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>94</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>104</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>114</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>117</v>
+      </c>
+      <c r="E300" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7306,7 +7856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7319,14 +7869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:38:48</t>
+          <t>Última actualización: 18:26:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -8135,7 +8685,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8149,9 +8699,59 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:42</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>76</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>117</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8168,7 +8768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8181,14 +8781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:38:48</t>
+          <t>Última actualización: 18:26:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -9022,7 +9622,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -9036,7 +9636,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -9066,6 +9666,56 @@
       <c r="E39" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>45</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>19:48</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>82</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2610
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E300"/>
+  <dimension ref="A1:E317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:26:37</t>
+          <t>Última actualización: 19:04:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 295</t>
+          <t>Total filas: 312</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>104</v>
+        <v>17</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>18</v>
+        <v>105</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3808,11 +3808,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>105</v>
+        <v>18</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>19:10</t>
+          <t>19:06</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7503,16 +7503,16 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>110</v>
+        <v>12</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>118</v>
+        <v>16</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>19:42</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7653,16 +7653,16 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>19:51</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7703,16 +7703,16 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>19:52</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,12 +7723,12 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>19:59</t>
+          <t>19:28</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>114</v>
+        <v>31</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,23 +7823,448 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
+          <t>17:38:48</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>118</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>19:42</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>38</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>39</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
           <t>18:26:37</t>
         </is>
       </c>
-      <c r="B300" t="inlineStr">
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>80</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>46</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>85</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>18:26:37</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>19:52</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>86</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>19:59</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>55</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>56</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>20:08</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>64</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>66</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>76</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>76</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
         <is>
           <t>20:23</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr">
+      <c r="C313" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D300" t="n">
-        <v>117</v>
-      </c>
-      <c r="E300" t="inlineStr">
+      <c r="D313" t="n">
+        <v>79</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>83</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>20:31</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>87</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>20:37</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>93</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>112</v>
+      </c>
+      <c r="E317" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7869,7 +8294,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:26:37</t>
+          <t>Última actualización: 19:04:56</t>
         </is>
       </c>
     </row>
@@ -8710,7 +9135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -8724,7 +9149,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -8735,7 +9160,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8749,7 +9174,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -8768,7 +9193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8781,14 +9206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:26:37</t>
+          <t>Última actualización: 19:04:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -9647,7 +10072,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -9661,7 +10086,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -9716,6 +10141,56 @@
       <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>45</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>101</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2611
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E317"/>
+  <dimension ref="A1:E337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:04:56</t>
+          <t>Última actualización: 19:53:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 312</t>
+          <t>Total filas: 332</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>105</v>
+        <v>18</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3808,11 +3808,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>18</v>
+        <v>105</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>14:43:05</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>14:43:05</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7483,11 +7483,11 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -7508,11 +7508,11 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7998,21 +7998,21 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>19:59</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>20:08</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,21 +8098,21 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>76</v>
+        <v>7</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>20:08</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:09</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,21 +8173,21 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>20:31</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>20:37</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>93</v>
+        <v>22</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,23 +8248,523 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>25</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>20:19</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>26</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
           <t>19:04:56</t>
         </is>
       </c>
-      <c r="B317" t="inlineStr">
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>76</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>76</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>28</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>30</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>83</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>20:28</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>35</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>20:31</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>87</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>20:32</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>39</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>20:37</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>44</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>52</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>55</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>20:52</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>59</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>19:04:56</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C317" t="inlineStr">
+      <c r="C331" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D317" t="n">
+      <c r="D331" t="n">
         <v>112</v>
       </c>
-      <c r="E317" t="inlineStr">
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>21:04</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>71</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>75</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>21:21</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>88</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>93</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>21:38</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>105</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>21:47</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>114</v>
+      </c>
+      <c r="E337" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8281,7 +8781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8294,14 +8794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:04:56</t>
+          <t>Última actualización: 19:53:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9660,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -9174,9 +9674,59 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>75</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>21:47</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>114</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9193,7 +9743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9206,14 +9756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:04:56</t>
+          <t>Última actualización: 19:53:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -10191,6 +10741,56 @@
       <c r="E43" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>20:46</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>53</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>21:29</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>96</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2612
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E337"/>
+  <dimension ref="A1:E356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:53:28</t>
+          <t>Última actualización: 20:26:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 332</t>
+          <t>Total filas: 351</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>104</v>
+        <v>17</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>10</v>
+        <v>76</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7483,11 +7483,11 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -7508,11 +7508,11 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7633,7 +7633,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D315" t="n">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D316" t="n">
@@ -8398,21 +8398,21 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,12 +8423,12 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>20:28</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -8437,7 +8437,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8453,16 +8453,16 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>20:31</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8478,16 +8478,16 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:28</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8498,21 +8498,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>20:37</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8528,16 +8528,16 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>20:48</t>
+          <t>20:37</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>20:52</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,21 +8598,21 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>112</v>
+        <v>52</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,21 +8623,21 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>21:04</t>
+          <t>20:47</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8653,16 +8653,16 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>21:08</t>
+          <t>20:48</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,21 +8673,21 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>21:21</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>88</v>
+        <v>26</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>93</v>
+        <v>26</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>21:38</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,23 +8748,498 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>31</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>35</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>21:04</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>38</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>41</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
           <t>19:53:28</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>75</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>42</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>54</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>21:21</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>88</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>21:22</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>56</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>21:22</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>56</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>93</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>71</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>71</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>21:38</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>105</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>80</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
         <is>
           <t>21:47</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C352" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D337" t="n">
+      <c r="D352" t="n">
         <v>114</v>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>93</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>101</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>106</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>22:18</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>112</v>
+      </c>
+      <c r="E356" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8781,7 +9256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8794,14 +9269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:53:28</t>
+          <t>Última actualización: 20:26:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -9685,12 +10160,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>21:08</t>
+          <t>21:07</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -9699,7 +10174,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -9715,18 +10190,68 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>75</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>80</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>19:53:28</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>21:47</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D43" t="n">
         <v>114</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9743,7 +10268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9756,14 +10281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:53:28</t>
+          <t>Última actualización: 20:26:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -10722,7 +11247,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10736,7 +11261,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -10772,25 +11297,100 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>21:28</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>62</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>19:53:28</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>21:29</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="D46" t="n">
         <v>96</v>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>101</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>22:20</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>114</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2613
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E356"/>
+  <dimension ref="A1:E370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:26:56</t>
+          <t>Última actualización: 20:58:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 351</t>
+          <t>Total filas: 365</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3698,7 +3698,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>11:21:53</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>17</v>
+        <v>104</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:21:53</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>104</v>
+        <v>17</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6783,7 +6783,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8773,12 +8773,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>21:04</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,21 +8823,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>21:07</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>21:08</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>21:08</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>21:04</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>54</v>
+        <v>6</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>21:21</t>
+          <t>21:07</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>88</v>
+        <v>9</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>21:22</t>
+          <t>21:08</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8978,16 +8978,16 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>21:22</t>
+          <t>21:08</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:20</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>93</v>
+        <v>22</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,21 +9023,21 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:21</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9053,16 +9053,16 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,21 +9073,21 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>21:38</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>105</v>
+        <v>24</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,21 +9098,21 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,21 +9123,21 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>21:47</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,21 +9148,21 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,12 +9173,12 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>19:53:28</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>22:07</t>
+          <t>21:38</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -9187,7 +9187,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9203,16 +9203,16 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>22:12</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,23 +9223,373 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>21:47</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>49</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>21:51</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>53</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
           <t>20:26:56</t>
         </is>
       </c>
-      <c r="B356" t="inlineStr">
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>93</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>62</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>69</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>70</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>106</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>20:26:56</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
         <is>
           <t>22:18</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr">
+      <c r="C363" t="inlineStr">
         <is>
           <t>26_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D356" t="n">
+      <c r="D363" t="n">
         <v>112</v>
       </c>
-      <c r="E356" t="inlineStr">
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>81</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>84</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>87</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>89</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>22:39</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>101</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>22:44</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>106</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>22:48</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>110</v>
+      </c>
+      <c r="E370" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9256,7 +9606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9269,14 +9619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:26:56</t>
+          <t>Última actualización: 20:58:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -10160,7 +10510,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10174,7 +10524,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -10235,7 +10585,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19:53:28</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10249,9 +10599,34 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20:58:45</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>22:39</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>101</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10281,7 +10656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:26:56</t>
+          <t>Última actualización: 20:58:45</t>
         </is>
       </c>
     </row>
@@ -11297,7 +11672,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -11311,7 +11686,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -11347,7 +11722,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -11361,7 +11736,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -11372,7 +11747,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -11386,7 +11761,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2614
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-21.xlsx
+++ b/data/horarios-141-2026-04-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E370"/>
+  <dimension ref="A1:E374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:58:45</t>
+          <t>Última actualización: 23:25:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 365</t>
+          <t>Total filas: 369</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:40:17</t>
+          <t>08:43:14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:43:14</t>
+          <t>07:40:17</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>13:42:48</t>
+          <t>12:48:15</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:48:15</t>
+          <t>13:42:48</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:51:15</t>
+          <t>15:45:19</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>10</v>
+        <v>76</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>15:45:19</t>
+          <t>16:51:15</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>17:38:48</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>17:38:48</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>19:04:56</t>
+          <t>18:26:37</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7483,11 +7483,11 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>18:26:37</t>
+          <t>19:04:56</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -7508,11 +7508,11 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D323" t="n">
@@ -8433,7 +8433,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D324" t="n">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8783,7 +8783,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D338" t="n">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D339" t="n">
@@ -8848,7 +8848,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>20:26:56</t>
+          <t>20:58:45</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -8858,11 +8858,11 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,7 +8873,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>20:58:45</t>
+          <t>20:26:56</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -8883,11 +8883,11 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -9590,6 +9590,106 @@
         <v>110</v>
       </c>
       <c r="E370" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>23:25:07</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>23:38</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>13</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>23:25:07</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>23:46</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>21</v>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>23:25:07</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>23:49</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>24</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>23:25:07</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>23:52</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>27</v>
+      </c>
+      <c r="E374" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9606,7 +9706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9619,14 +9719,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:58:45</t>
+          <t>Última actualización: 23:25:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -10627,6 +10727,31 @@
         <v>101</v>
       </c>
       <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>23:25:07</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>23:38</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>13</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10656,7 +10781,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:58:45</t>
+          <t>Última actualización: 23:25:07</t>
         </is>
       </c>
     </row>

</xml_diff>